<commit_message>
PDF for shader summary
</commit_message>
<xml_diff>
--- a/Documentation/Shaders-Summary.xlsx
+++ b/Documentation/Shaders-Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qesrg\Desktop\CG\3D-Data-Visualizer\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BE8AA3-51D2-4845-8B64-D001456794B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E36776BE-14C9-4449-894B-877BDCBD3303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{21468231-176E-4380-A623-6D9DD4C234A8}"/>
   </bookViews>
@@ -591,6 +591,48 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -613,48 +655,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1092,6 +1092,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1983EE3C-D493-4059-B49D-A64E57E2F103}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:G36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1106,22 +1109,22 @@
   <sheetData>
     <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="36"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="32"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="37"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
-      <c r="G3" s="39"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="35"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1455,22 +1458,22 @@
       <c r="G23" s="4"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B24" s="34" t="s">
+      <c r="B24" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="36"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="32"/>
     </row>
     <row r="25" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="37"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="39"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="35"/>
     </row>
     <row r="26" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
@@ -1482,12 +1485,12 @@
     </row>
     <row r="27" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
-      <c r="C27" s="40" t="s">
+      <c r="C27" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
       <c r="G27" s="7" t="s">
         <v>67</v>
       </c>
@@ -1496,12 +1499,12 @@
       <c r="B28" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="42" t="s">
+      <c r="C28" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="D28" s="43"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="39"/>
       <c r="G28" s="19" t="s">
         <v>78</v>
       </c>
@@ -1510,12 +1513,12 @@
       <c r="B29" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C29" s="44" t="s">
+      <c r="C29" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="45"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
       <c r="G29" s="15" t="s">
         <v>79</v>
       </c>
@@ -1524,12 +1527,12 @@
       <c r="B30" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="46" t="s">
+      <c r="C30" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="21" t="s">
         <v>80</v>
       </c>
@@ -1538,12 +1541,12 @@
       <c r="B31" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="44" t="s">
+      <c r="C31" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
       <c r="G31" s="15" t="s">
         <v>81</v>
       </c>
@@ -1552,12 +1555,12 @@
       <c r="B32" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="C32" s="26" t="s">
+      <c r="C32" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
       <c r="G32" s="23" t="s">
         <v>82</v>
       </c>
@@ -1566,12 +1569,12 @@
       <c r="B33" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
+      <c r="D33" s="43"/>
+      <c r="E33" s="43"/>
+      <c r="F33" s="43"/>
       <c r="G33" s="15" t="s">
         <v>83</v>
       </c>
@@ -1580,12 +1583,12 @@
       <c r="B34" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="30" t="s">
+      <c r="C34" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
+      <c r="D34" s="45"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="45"/>
       <c r="G34" s="21" t="s">
         <v>84</v>
       </c>
@@ -1594,12 +1597,12 @@
       <c r="B35" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
-      <c r="F35" s="29"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
       <c r="G35" s="15" t="s">
         <v>85</v>
       </c>
@@ -1608,18 +1611,23 @@
       <c r="B36" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="32" t="s">
+      <c r="C36" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
+      <c r="F36" s="47"/>
       <c r="G36" s="25" t="s">
         <v>86</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
     <mergeCell ref="C30:F30"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="B24:G25"/>
@@ -1627,15 +1635,11 @@
     <mergeCell ref="C27:F27"/>
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="59" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>